<commit_message>
updated on 1 SEP
</commit_message>
<xml_diff>
--- a/CAP776 (PYTHON).xlsx
+++ b/CAP776 (PYTHON).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\palak\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\palak\Downloads\776(clone)\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2536E73-460D-4FC2-8B44-B8A788EA2FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51051FB3-5E3F-4E8D-AB35-96B05F7E0056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{327CE7B2-1886-45B8-951C-28CB36CE6AAF}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="40">
   <si>
     <t>My Data, My Code — Daily Log</t>
   </si>
@@ -137,6 +137,24 @@
   <si>
     <t>Relaxed</t>
   </si>
+  <si>
+    <t>Busy</t>
+  </si>
+  <si>
+    <t>Heavy travel &amp; long class day</t>
+  </si>
+  <si>
+    <t>Managed classes, self-study</t>
+  </si>
+  <si>
+    <t>Moderate class schedule with coding focus</t>
+  </si>
+  <si>
+    <t>Exhausted</t>
+  </si>
+  <si>
+    <t>Full lecture day with heavy travel schedule</t>
+  </si>
 </sst>
 </file>
 
@@ -145,7 +163,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +220,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -223,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -246,12 +270,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -288,9 +327,22 @@
     <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E7F1806-3D91-4029-8849-359DB02F0997}">
-  <dimension ref="A1:N377"/>
+  <dimension ref="A1:O376"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.21875" customWidth="1"/>
@@ -626,39 +678,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="18">
         <v>12617802</v>
       </c>
-      <c r="G2" s="16"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -671,18 +723,18 @@
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
       <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="16"/>
+      <c r="G3" s="18"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -692,22 +744,22 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
     </row>
     <row r="5" spans="1:14" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1215,7 +1267,7 @@
       </c>
       <c r="N16" s="10"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="12">
         <v>46257</v>
       </c>
@@ -1257,8 +1309,8 @@
       </c>
       <c r="N17" s="10"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="12">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18" s="19">
         <v>46258</v>
       </c>
       <c r="B18" s="10">
@@ -1297,53 +1349,144 @@
       <c r="M18" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="N18" s="10"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="4" t="str">
-        <f t="shared" ref="I20:I44" si="0">IF(SUM(B20:F20,H20)=0,"",SUM(B20:F20,H20))</f>
-        <v/>
-      </c>
-      <c r="J20" s="4" t="str">
-        <f t="shared" ref="J20:J44" si="1">IF(I20="","",1440-I20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="8"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="8"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N18" t="s">
+        <v>36</v>
+      </c>
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="12">
+        <v>46259</v>
+      </c>
+      <c r="B19" s="10">
+        <v>360</v>
+      </c>
+      <c r="C19" s="10">
+        <v>30</v>
+      </c>
+      <c r="D19" s="10">
+        <v>120</v>
+      </c>
+      <c r="E19" s="10">
+        <v>120</v>
+      </c>
+      <c r="F19" s="10">
+        <v>350</v>
+      </c>
+      <c r="G19" s="10">
+        <v>7</v>
+      </c>
+      <c r="H19" s="10">
+        <v>360</v>
+      </c>
+      <c r="I19" s="10">
+        <v>1340</v>
+      </c>
+      <c r="J19" s="10">
+        <v>100</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="N19" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="12">
+        <v>46260</v>
+      </c>
+      <c r="B20" s="15">
+        <v>360</v>
+      </c>
+      <c r="C20" s="20">
+        <v>45</v>
+      </c>
+      <c r="D20" s="20">
+        <v>150</v>
+      </c>
+      <c r="E20" s="20">
+        <v>150</v>
+      </c>
+      <c r="F20" s="20">
+        <v>200</v>
+      </c>
+      <c r="G20" s="20">
+        <v>4</v>
+      </c>
+      <c r="H20" s="20">
+        <v>240</v>
+      </c>
+      <c r="I20" s="20">
+        <v>1145</v>
+      </c>
+      <c r="J20" s="20">
+        <v>295</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="M20" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="N20" s="14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="12">
+        <v>46261</v>
+      </c>
+      <c r="B21" s="21">
+        <v>360</v>
+      </c>
+      <c r="C21" s="21">
+        <v>30</v>
+      </c>
+      <c r="D21" s="21">
+        <v>90</v>
+      </c>
+      <c r="E21" s="21">
+        <v>120</v>
+      </c>
+      <c r="F21" s="21">
+        <v>400</v>
+      </c>
+      <c r="G21" s="21">
+        <v>8</v>
+      </c>
+      <c r="H21" s="21">
+        <v>300</v>
+      </c>
+      <c r="I21" s="21">
+        <v>1300</v>
+      </c>
+      <c r="J21" s="21">
+        <v>140</v>
+      </c>
+      <c r="K21" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="L21" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" s="14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1353,11 +1496,11 @@
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="I22:I43" si="0">IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
         <v/>
       </c>
       <c r="J22" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J22:J43" si="1">IF(I22="","",1440-I22)</f>
         <v/>
       </c>
       <c r="K22" s="7"/>
@@ -1365,7 +1508,7 @@
       <c r="M22" s="7"/>
       <c r="N22" s="8"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1387,7 +1530,7 @@
       <c r="M23" s="7"/>
       <c r="N23" s="8"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1409,7 +1552,7 @@
       <c r="M24" s="7"/>
       <c r="N24" s="8"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1431,7 +1574,7 @@
       <c r="M25" s="7"/>
       <c r="N25" s="8"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1453,7 +1596,7 @@
       <c r="M26" s="7"/>
       <c r="N26" s="8"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1475,7 +1618,7 @@
       <c r="M27" s="7"/>
       <c r="N27" s="8"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1497,7 +1640,7 @@
       <c r="M28" s="7"/>
       <c r="N28" s="8"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1519,7 +1662,7 @@
       <c r="M29" s="7"/>
       <c r="N29" s="8"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1541,7 +1684,7 @@
       <c r="M30" s="7"/>
       <c r="N30" s="8"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1563,7 +1706,7 @@
       <c r="M31" s="7"/>
       <c r="N31" s="8"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="5"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1837,11 +1980,11 @@
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
       <c r="I44" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="I44:I107" si="2">IF(SUM(B44:F44,H44)=0,"",SUM(B44:F44,H44))</f>
         <v/>
       </c>
       <c r="J44" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J44:J107" si="3">IF(I44="","",1440-I44)</f>
         <v/>
       </c>
       <c r="K44" s="7"/>
@@ -1859,11 +2002,11 @@
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
       <c r="I45" s="4" t="str">
-        <f t="shared" ref="I45:I108" si="2">IF(SUM(B45:F45,H45)=0,"",SUM(B45:F45,H45))</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="J45" s="4" t="str">
-        <f t="shared" ref="J45:J108" si="3">IF(I45="","",1440-I45)</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K45" s="7"/>
@@ -3245,11 +3388,11 @@
       <c r="G108" s="6"/>
       <c r="H108" s="6"/>
       <c r="I108" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I108:I171" si="4">IF(SUM(B108:F108,H108)=0,"",SUM(B108:F108,H108))</f>
         <v/>
       </c>
       <c r="J108" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J108:J171" si="5">IF(I108="","",1440-I108)</f>
         <v/>
       </c>
       <c r="K108" s="7"/>
@@ -3267,11 +3410,11 @@
       <c r="G109" s="6"/>
       <c r="H109" s="6"/>
       <c r="I109" s="4" t="str">
-        <f t="shared" ref="I109:I172" si="4">IF(SUM(B109:F109,H109)=0,"",SUM(B109:F109,H109))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J109" s="4" t="str">
-        <f t="shared" ref="J109:J172" si="5">IF(I109="","",1440-I109)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K109" s="7"/>
@@ -4653,11 +4796,11 @@
       <c r="G172" s="6"/>
       <c r="H172" s="6"/>
       <c r="I172" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I172:I235" si="6">IF(SUM(B172:F172,H172)=0,"",SUM(B172:F172,H172))</f>
         <v/>
       </c>
       <c r="J172" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="J172:J235" si="7">IF(I172="","",1440-I172)</f>
         <v/>
       </c>
       <c r="K172" s="7"/>
@@ -4675,11 +4818,11 @@
       <c r="G173" s="6"/>
       <c r="H173" s="6"/>
       <c r="I173" s="4" t="str">
-        <f t="shared" ref="I173:I236" si="6">IF(SUM(B173:F173,H173)=0,"",SUM(B173:F173,H173))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J173" s="4" t="str">
-        <f t="shared" ref="J173:J236" si="7">IF(I173="","",1440-I173)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K173" s="7"/>
@@ -6061,11 +6204,11 @@
       <c r="G236" s="6"/>
       <c r="H236" s="6"/>
       <c r="I236" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I236:I299" si="8">IF(SUM(B236:F236,H236)=0,"",SUM(B236:F236,H236))</f>
         <v/>
       </c>
       <c r="J236" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="J236:J299" si="9">IF(I236="","",1440-I236)</f>
         <v/>
       </c>
       <c r="K236" s="7"/>
@@ -6083,11 +6226,11 @@
       <c r="G237" s="6"/>
       <c r="H237" s="6"/>
       <c r="I237" s="4" t="str">
-        <f t="shared" ref="I237:I300" si="8">IF(SUM(B237:F237,H237)=0,"",SUM(B237:F237,H237))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J237" s="4" t="str">
-        <f t="shared" ref="J237:J300" si="9">IF(I237="","",1440-I237)</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K237" s="7"/>
@@ -7469,11 +7612,11 @@
       <c r="G300" s="6"/>
       <c r="H300" s="6"/>
       <c r="I300" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I300:I363" si="10">IF(SUM(B300:F300,H300)=0,"",SUM(B300:F300,H300))</f>
         <v/>
       </c>
       <c r="J300" s="4" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="J300:J363" si="11">IF(I300="","",1440-I300)</f>
         <v/>
       </c>
       <c r="K300" s="7"/>
@@ -7491,11 +7634,11 @@
       <c r="G301" s="6"/>
       <c r="H301" s="6"/>
       <c r="I301" s="4" t="str">
-        <f t="shared" ref="I301:I364" si="10">IF(SUM(B301:F301,H301)=0,"",SUM(B301:F301,H301))</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J301" s="4" t="str">
-        <f t="shared" ref="J301:J364" si="11">IF(I301="","",1440-I301)</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K301" s="7"/>
@@ -8877,11 +9020,11 @@
       <c r="G364" s="6"/>
       <c r="H364" s="6"/>
       <c r="I364" s="4" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I364:I376" si="12">IF(SUM(B364:F364,H364)=0,"",SUM(B364:F364,H364))</f>
         <v/>
       </c>
       <c r="J364" s="4" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="J364:J376" si="13">IF(I364="","",1440-I364)</f>
         <v/>
       </c>
       <c r="K364" s="7"/>
@@ -8899,11 +9042,11 @@
       <c r="G365" s="6"/>
       <c r="H365" s="6"/>
       <c r="I365" s="4" t="str">
-        <f t="shared" ref="I365:I377" si="12">IF(SUM(B365:F365,H365)=0,"",SUM(B365:F365,H365))</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J365" s="4" t="str">
-        <f t="shared" ref="J365:J377" si="13">IF(I365="","",1440-I365)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K365" s="7"/>
@@ -9110,14 +9253,6 @@
       <c r="N374" s="8"/>
     </row>
     <row r="375" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A375" s="5"/>
-      <c r="B375" s="6"/>
-      <c r="C375" s="6"/>
-      <c r="D375" s="6"/>
-      <c r="E375" s="6"/>
-      <c r="F375" s="6"/>
-      <c r="G375" s="6"/>
-      <c r="H375" s="6"/>
       <c r="I375" s="4" t="str">
         <f t="shared" si="12"/>
         <v/>
@@ -9126,10 +9261,6 @@
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="K375" s="7"/>
-      <c r="L375" s="7"/>
-      <c r="M375" s="7"/>
-      <c r="N375" s="8"/>
     </row>
     <row r="376" spans="1:14" x14ac:dyDescent="0.3">
       <c r="I376" s="4" t="str">
@@ -9137,16 +9268,6 @@
         <v/>
       </c>
       <c r="J376" s="4" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-    </row>
-    <row r="377" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="I377" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="J377" s="4" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>

</xml_diff>